<commit_message>
feat: update scoring table to August revision
</commit_message>
<xml_diff>
--- a/DOC/AI 测评 访谈及报告流程/000 10题赋分.xlsx
+++ b/DOC/AI 测评 访谈及报告流程/000 10题赋分.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23837" windowHeight="12548"/>
+    <workbookView windowHeight="17655"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,20 +33,12 @@
   </si>
   <si>
     <r>
+      <t>第</t>
+    </r>
+    <r>
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>第</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
         <charset val="134"/>
       </rPr>
@@ -56,7 +48,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -66,7 +57,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
@@ -81,7 +71,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -91,7 +80,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
@@ -106,7 +94,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -116,7 +103,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
@@ -131,7 +117,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -141,7 +126,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
@@ -150,20 +134,12 @@
   </si>
   <si>
     <r>
+      <t>第</t>
+    </r>
+    <r>
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>第</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
         <charset val="134"/>
       </rPr>
@@ -173,7 +149,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -183,7 +158,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
@@ -198,7 +172,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -208,7 +181,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
@@ -223,7 +195,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -233,7 +204,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
@@ -251,7 +221,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -261,7 +230,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
@@ -276,7 +244,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -286,7 +253,6 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
@@ -400,7 +366,6 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="宋体-简"/>
       <charset val="134"/>
     </font>
@@ -409,13 +374,6 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -564,23 +522,22 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -910,52 +867,55 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -970,77 +930,74 @@
     <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1053,25 +1010,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1600,14 +1545,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:K25"/>
-  <sheetFormatPr defaultColWidth="9.23423423423423" defaultRowHeight="15.4"/>
+  <sheetFormatPr defaultColWidth="9.23333333333333" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="14.7207207207207" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.8918918918919" style="1" customWidth="1"/>
-    <col min="3" max="11" width="11.8918918918919" style="2" customWidth="1"/>
+    <col min="1" max="1" width="14.7166666666667" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.8916666666667" style="1" customWidth="1"/>
+    <col min="3" max="11" width="11.8916666666667" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" spans="1:11">
+    <row r="1" spans="1:11">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1649,32 +1594,32 @@
       <c r="B2" s="6">
         <v>4</v>
       </c>
-      <c r="C2" s="7">
-        <v>2</v>
-      </c>
-      <c r="D2" s="8">
-        <v>2</v>
-      </c>
-      <c r="E2" s="9">
-        <v>0</v>
-      </c>
-      <c r="F2" s="10">
-        <v>3</v>
+      <c r="C2" s="6">
+        <v>2</v>
+      </c>
+      <c r="D2" s="6">
+        <v>0</v>
+      </c>
+      <c r="E2" s="6">
+        <v>3</v>
+      </c>
+      <c r="F2" s="6">
+        <v>2</v>
       </c>
       <c r="G2" s="6">
         <v>0</v>
       </c>
-      <c r="H2" s="9">
-        <v>0</v>
-      </c>
-      <c r="I2" s="7">
-        <v>1</v>
-      </c>
-      <c r="J2" s="9">
-        <v>0</v>
-      </c>
-      <c r="K2" s="7">
-        <v>2</v>
+      <c r="H2" s="6">
+        <v>2</v>
+      </c>
+      <c r="I2" s="6">
+        <v>1</v>
+      </c>
+      <c r="J2" s="6">
+        <v>1</v>
+      </c>
+      <c r="K2" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1684,31 +1629,31 @@
       <c r="B3" s="6">
         <v>3</v>
       </c>
-      <c r="C3" s="7">
-        <v>2</v>
-      </c>
-      <c r="D3" s="8">
-        <v>4</v>
-      </c>
-      <c r="E3" s="9">
-        <v>2</v>
-      </c>
-      <c r="F3" s="10">
+      <c r="C3" s="6">
+        <v>2</v>
+      </c>
+      <c r="D3" s="6">
+        <v>0</v>
+      </c>
+      <c r="E3" s="6">
+        <v>3</v>
+      </c>
+      <c r="F3" s="6">
         <v>2</v>
       </c>
       <c r="G3" s="6">
         <v>0</v>
       </c>
-      <c r="H3" s="9">
-        <v>1</v>
-      </c>
-      <c r="I3" s="7">
-        <v>2</v>
-      </c>
-      <c r="J3" s="9">
-        <v>3</v>
-      </c>
-      <c r="K3" s="7">
+      <c r="H3" s="6">
+        <v>2</v>
+      </c>
+      <c r="I3" s="6">
+        <v>1</v>
+      </c>
+      <c r="J3" s="6">
+        <v>0</v>
+      </c>
+      <c r="K3" s="6">
         <v>2</v>
       </c>
     </row>
@@ -1719,31 +1664,31 @@
       <c r="B4" s="6">
         <v>4</v>
       </c>
-      <c r="C4" s="7">
-        <v>3</v>
-      </c>
-      <c r="D4" s="8">
-        <v>1</v>
-      </c>
-      <c r="E4" s="9">
-        <v>1</v>
-      </c>
-      <c r="F4" s="10">
-        <v>3</v>
+      <c r="C4" s="6">
+        <v>3</v>
+      </c>
+      <c r="D4" s="6">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6">
+        <v>2</v>
+      </c>
+      <c r="F4" s="6">
+        <v>2</v>
       </c>
       <c r="G4" s="6">
         <v>0</v>
       </c>
-      <c r="H4" s="9">
-        <v>1</v>
-      </c>
-      <c r="I4" s="7">
-        <v>2</v>
-      </c>
-      <c r="J4" s="9">
-        <v>0</v>
-      </c>
-      <c r="K4" s="7">
+      <c r="H4" s="6">
+        <v>3</v>
+      </c>
+      <c r="I4" s="6">
+        <v>1</v>
+      </c>
+      <c r="J4" s="6">
+        <v>0</v>
+      </c>
+      <c r="K4" s="6">
         <v>1</v>
       </c>
     </row>
@@ -1754,31 +1699,31 @@
       <c r="B5" s="6">
         <v>2</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>4</v>
       </c>
-      <c r="D5" s="8">
-        <v>1</v>
-      </c>
-      <c r="E5" s="9">
-        <v>1</v>
-      </c>
-      <c r="F5" s="10">
+      <c r="D5" s="6">
+        <v>2</v>
+      </c>
+      <c r="E5" s="6">
+        <v>1</v>
+      </c>
+      <c r="F5" s="6">
         <v>1</v>
       </c>
       <c r="G5" s="6">
         <v>0</v>
       </c>
-      <c r="H5" s="9">
-        <v>1</v>
-      </c>
-      <c r="I5" s="7">
-        <v>2</v>
-      </c>
-      <c r="J5" s="9">
-        <v>1</v>
-      </c>
-      <c r="K5" s="7">
+      <c r="H5" s="6">
+        <v>2</v>
+      </c>
+      <c r="I5" s="6">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6">
+        <v>1</v>
+      </c>
+      <c r="K5" s="6">
         <v>1</v>
       </c>
     </row>
@@ -1789,32 +1734,32 @@
       <c r="B6" s="6">
         <v>1</v>
       </c>
-      <c r="C6" s="7">
-        <v>2</v>
-      </c>
-      <c r="D6" s="8">
-        <v>4</v>
-      </c>
-      <c r="E6" s="9">
-        <v>1</v>
-      </c>
-      <c r="F6" s="10">
+      <c r="C6" s="6">
+        <v>2</v>
+      </c>
+      <c r="D6" s="6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="6">
+        <v>2</v>
+      </c>
+      <c r="F6" s="6">
         <v>1</v>
       </c>
       <c r="G6" s="6">
         <v>0</v>
       </c>
-      <c r="H6" s="9">
-        <v>1</v>
-      </c>
-      <c r="I6" s="7">
-        <v>2</v>
-      </c>
-      <c r="J6" s="9">
-        <v>2</v>
-      </c>
-      <c r="K6" s="7">
-        <v>2</v>
+      <c r="H6" s="6">
+        <v>0</v>
+      </c>
+      <c r="I6" s="6">
+        <v>1</v>
+      </c>
+      <c r="J6" s="6">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1824,32 +1769,32 @@
       <c r="B7" s="6">
         <v>1</v>
       </c>
-      <c r="C7" s="7">
-        <v>3</v>
-      </c>
-      <c r="D7" s="8">
-        <v>3</v>
-      </c>
-      <c r="E7" s="9">
-        <v>2</v>
-      </c>
-      <c r="F7" s="10">
+      <c r="C7" s="6">
+        <v>3</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6">
+        <v>1</v>
+      </c>
+      <c r="F7" s="6">
         <v>0</v>
       </c>
       <c r="G7" s="6">
         <v>1</v>
       </c>
-      <c r="H7" s="9">
-        <v>3</v>
-      </c>
-      <c r="I7" s="7">
-        <v>3</v>
-      </c>
-      <c r="J7" s="9">
-        <v>1</v>
-      </c>
-      <c r="K7" s="7">
-        <v>1</v>
+      <c r="H7" s="6">
+        <v>1</v>
+      </c>
+      <c r="I7" s="6">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6">
+        <v>1</v>
+      </c>
+      <c r="K7" s="6">
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1859,32 +1804,32 @@
       <c r="B8" s="6">
         <v>2</v>
       </c>
-      <c r="C8" s="7">
-        <v>2</v>
-      </c>
-      <c r="D8" s="8">
-        <v>2</v>
-      </c>
-      <c r="E8" s="9">
-        <v>1</v>
-      </c>
-      <c r="F8" s="10">
+      <c r="C8" s="6">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6">
+        <v>0</v>
+      </c>
+      <c r="E8" s="6">
+        <v>4</v>
+      </c>
+      <c r="F8" s="6">
         <v>3</v>
       </c>
       <c r="G8" s="6">
         <v>0</v>
       </c>
-      <c r="H8" s="9">
-        <v>0</v>
-      </c>
-      <c r="I8" s="7">
-        <v>1</v>
-      </c>
-      <c r="J8" s="9">
-        <v>2</v>
-      </c>
-      <c r="K8" s="7">
-        <v>2</v>
+      <c r="H8" s="6">
+        <v>2</v>
+      </c>
+      <c r="I8" s="6">
+        <v>2</v>
+      </c>
+      <c r="J8" s="6">
+        <v>2</v>
+      </c>
+      <c r="K8" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1894,32 +1839,32 @@
       <c r="B9" s="6">
         <v>1</v>
       </c>
-      <c r="C9" s="7">
-        <v>1</v>
-      </c>
-      <c r="D9" s="8">
-        <v>2</v>
-      </c>
-      <c r="E9" s="9">
+      <c r="C9" s="6">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6">
+        <v>0</v>
+      </c>
+      <c r="E9" s="6">
+        <v>3</v>
+      </c>
+      <c r="F9" s="6">
+        <v>3</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6">
+        <v>1</v>
+      </c>
+      <c r="I9" s="6">
+        <v>2</v>
+      </c>
+      <c r="J9" s="6">
+        <v>2</v>
+      </c>
+      <c r="K9" s="6">
         <v>4</v>
-      </c>
-      <c r="F9" s="10">
-        <v>4</v>
-      </c>
-      <c r="G9" s="6">
-        <v>0</v>
-      </c>
-      <c r="H9" s="9">
-        <v>2</v>
-      </c>
-      <c r="I9" s="7">
-        <v>1</v>
-      </c>
-      <c r="J9" s="9">
-        <v>2</v>
-      </c>
-      <c r="K9" s="7">
-        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1929,31 +1874,31 @@
       <c r="B10" s="6">
         <v>3</v>
       </c>
-      <c r="C10" s="7">
-        <v>1</v>
-      </c>
-      <c r="D10" s="8">
-        <v>4</v>
-      </c>
-      <c r="E10" s="9">
-        <v>2</v>
-      </c>
-      <c r="F10" s="10">
+      <c r="C10" s="6">
+        <v>1</v>
+      </c>
+      <c r="D10" s="6">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6">
+        <v>3</v>
+      </c>
+      <c r="F10" s="6">
         <v>2</v>
       </c>
       <c r="G10" s="6">
         <v>1</v>
       </c>
-      <c r="H10" s="9">
-        <v>1</v>
-      </c>
-      <c r="I10" s="7">
-        <v>0</v>
-      </c>
-      <c r="J10" s="9">
-        <v>1</v>
-      </c>
-      <c r="K10" s="7">
+      <c r="H10" s="6">
+        <v>2</v>
+      </c>
+      <c r="I10" s="6">
+        <v>3</v>
+      </c>
+      <c r="J10" s="6">
+        <v>2</v>
+      </c>
+      <c r="K10" s="6">
         <v>2</v>
       </c>
     </row>
@@ -1964,32 +1909,32 @@
       <c r="B11" s="6">
         <v>1</v>
       </c>
-      <c r="C11" s="7">
-        <v>1</v>
-      </c>
-      <c r="D11" s="8">
+      <c r="C11" s="6">
+        <v>1</v>
+      </c>
+      <c r="D11" s="6">
+        <v>1</v>
+      </c>
+      <c r="E11" s="6">
+        <v>2</v>
+      </c>
+      <c r="F11" s="6">
+        <v>1</v>
+      </c>
+      <c r="G11" s="6">
+        <v>3</v>
+      </c>
+      <c r="H11" s="6">
+        <v>1</v>
+      </c>
+      <c r="I11" s="6">
         <v>4</v>
       </c>
-      <c r="E11" s="9">
-        <v>3</v>
-      </c>
-      <c r="F11" s="10">
-        <v>1</v>
-      </c>
-      <c r="G11" s="6">
-        <v>3</v>
-      </c>
-      <c r="H11" s="9">
-        <v>1</v>
-      </c>
-      <c r="I11" s="7">
-        <v>1</v>
-      </c>
-      <c r="J11" s="9">
-        <v>0</v>
-      </c>
-      <c r="K11" s="7">
-        <v>2</v>
+      <c r="J11" s="6">
+        <v>3</v>
+      </c>
+      <c r="K11" s="6">
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1999,31 +1944,31 @@
       <c r="B12" s="6">
         <v>1</v>
       </c>
-      <c r="C12" s="7">
-        <v>1</v>
-      </c>
-      <c r="D12" s="8">
+      <c r="C12" s="6">
+        <v>1</v>
+      </c>
+      <c r="D12" s="6">
+        <v>2</v>
+      </c>
+      <c r="E12" s="6">
+        <v>2</v>
+      </c>
+      <c r="F12" s="6">
         <v>4</v>
       </c>
-      <c r="E12" s="9">
-        <v>4</v>
-      </c>
-      <c r="F12" s="10">
-        <v>3</v>
-      </c>
       <c r="G12" s="6">
         <v>2</v>
       </c>
-      <c r="H12" s="9">
-        <v>2</v>
-      </c>
-      <c r="I12" s="7">
-        <v>2</v>
-      </c>
-      <c r="J12" s="9">
-        <v>2</v>
-      </c>
-      <c r="K12" s="7">
+      <c r="H12" s="6">
+        <v>2</v>
+      </c>
+      <c r="I12" s="6">
+        <v>2</v>
+      </c>
+      <c r="J12" s="6">
+        <v>0</v>
+      </c>
+      <c r="K12" s="6">
         <v>4</v>
       </c>
     </row>
@@ -2034,32 +1979,32 @@
       <c r="B13" s="6">
         <v>0</v>
       </c>
-      <c r="C13" s="7">
-        <v>0</v>
-      </c>
-      <c r="D13" s="8">
-        <v>2</v>
-      </c>
-      <c r="E13" s="9">
+      <c r="C13" s="6">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6">
+        <v>2</v>
+      </c>
+      <c r="F13" s="6">
+        <v>3</v>
+      </c>
+      <c r="G13" s="6">
+        <v>3</v>
+      </c>
+      <c r="H13" s="6">
+        <v>1</v>
+      </c>
+      <c r="I13" s="6">
+        <v>3</v>
+      </c>
+      <c r="J13" s="6">
+        <v>0</v>
+      </c>
+      <c r="K13" s="6">
         <v>4</v>
-      </c>
-      <c r="F13" s="10">
-        <v>2</v>
-      </c>
-      <c r="G13" s="6">
-        <v>3</v>
-      </c>
-      <c r="H13" s="9">
-        <v>0</v>
-      </c>
-      <c r="I13" s="7">
-        <v>1</v>
-      </c>
-      <c r="J13" s="9">
-        <v>1</v>
-      </c>
-      <c r="K13" s="7">
-        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2069,31 +2014,31 @@
       <c r="B14" s="6">
         <v>4</v>
       </c>
-      <c r="C14" s="7">
-        <v>2</v>
-      </c>
-      <c r="D14" s="8">
-        <v>3</v>
-      </c>
-      <c r="E14" s="9">
-        <v>1</v>
-      </c>
-      <c r="F14" s="10">
+      <c r="C14" s="6">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6">
+        <v>1</v>
+      </c>
+      <c r="E14" s="6">
+        <v>2</v>
+      </c>
+      <c r="F14" s="6">
         <v>1</v>
       </c>
       <c r="G14" s="6">
         <v>1</v>
       </c>
-      <c r="H14" s="9">
-        <v>2</v>
-      </c>
-      <c r="I14" s="7">
-        <v>1</v>
-      </c>
-      <c r="J14" s="9">
-        <v>0</v>
-      </c>
-      <c r="K14" s="7">
+      <c r="H14" s="6">
+        <v>3</v>
+      </c>
+      <c r="I14" s="6">
+        <v>1</v>
+      </c>
+      <c r="J14" s="6">
+        <v>2</v>
+      </c>
+      <c r="K14" s="6">
         <v>1</v>
       </c>
     </row>
@@ -2104,32 +2049,32 @@
       <c r="B15" s="6">
         <v>2</v>
       </c>
-      <c r="C15" s="7">
-        <v>3</v>
-      </c>
-      <c r="D15" s="8">
-        <v>1</v>
-      </c>
-      <c r="E15" s="9">
-        <v>1</v>
-      </c>
-      <c r="F15" s="10">
+      <c r="C15" s="6">
+        <v>3</v>
+      </c>
+      <c r="D15" s="6">
+        <v>3</v>
+      </c>
+      <c r="E15" s="6">
+        <v>1</v>
+      </c>
+      <c r="F15" s="6">
         <v>0</v>
       </c>
       <c r="G15" s="6">
         <v>1</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="6">
         <v>4</v>
       </c>
-      <c r="I15" s="7">
-        <v>2</v>
-      </c>
-      <c r="J15" s="9">
-        <v>1</v>
-      </c>
-      <c r="K15" s="7">
-        <v>0</v>
+      <c r="I15" s="6">
+        <v>0</v>
+      </c>
+      <c r="J15" s="6">
+        <v>2</v>
+      </c>
+      <c r="K15" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -2139,32 +2084,32 @@
       <c r="B16" s="6">
         <v>3</v>
       </c>
-      <c r="C16" s="7">
-        <v>2</v>
-      </c>
-      <c r="D16" s="8">
-        <v>3</v>
-      </c>
-      <c r="E16" s="9">
-        <v>2</v>
-      </c>
-      <c r="F16" s="10">
+      <c r="C16" s="6">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6">
+        <v>2</v>
+      </c>
+      <c r="E16" s="6">
+        <v>2</v>
+      </c>
+      <c r="F16" s="6">
         <v>0</v>
       </c>
       <c r="G16" s="6">
         <v>2</v>
       </c>
-      <c r="H16" s="9">
-        <v>2</v>
-      </c>
-      <c r="I16" s="7">
-        <v>1</v>
-      </c>
-      <c r="J16" s="9">
-        <v>1</v>
-      </c>
-      <c r="K16" s="7">
-        <v>1</v>
+      <c r="H16" s="6">
+        <v>2</v>
+      </c>
+      <c r="I16" s="6">
+        <v>3</v>
+      </c>
+      <c r="J16" s="6">
+        <v>3</v>
+      </c>
+      <c r="K16" s="6">
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -2174,32 +2119,32 @@
       <c r="B17" s="6">
         <v>1</v>
       </c>
-      <c r="C17" s="7">
-        <v>1</v>
-      </c>
-      <c r="D17" s="8">
-        <v>1</v>
-      </c>
-      <c r="E17" s="9">
-        <v>1</v>
-      </c>
-      <c r="F17" s="10">
+      <c r="C17" s="6">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6">
+        <v>1</v>
+      </c>
+      <c r="E17" s="6">
+        <v>1</v>
+      </c>
+      <c r="F17" s="6">
         <v>1</v>
       </c>
       <c r="G17" s="6">
         <v>4</v>
       </c>
-      <c r="H17" s="9">
-        <v>2</v>
-      </c>
-      <c r="I17" s="7">
-        <v>1</v>
-      </c>
-      <c r="J17" s="9">
-        <v>0</v>
-      </c>
-      <c r="K17" s="7">
-        <v>2</v>
+      <c r="H17" s="6">
+        <v>1</v>
+      </c>
+      <c r="I17" s="6">
+        <v>3</v>
+      </c>
+      <c r="J17" s="6">
+        <v>2</v>
+      </c>
+      <c r="K17" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2209,32 +2154,32 @@
       <c r="B18" s="6">
         <v>2</v>
       </c>
-      <c r="C18" s="7">
-        <v>2</v>
-      </c>
-      <c r="D18" s="8">
-        <v>0</v>
-      </c>
-      <c r="E18" s="9">
-        <v>2</v>
-      </c>
-      <c r="F18" s="10">
-        <v>2</v>
+      <c r="C18" s="6">
+        <v>2</v>
+      </c>
+      <c r="D18" s="6">
+        <v>4</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6">
+        <v>1</v>
       </c>
       <c r="G18" s="6">
         <v>2</v>
       </c>
-      <c r="H18" s="9">
-        <v>4</v>
-      </c>
-      <c r="I18" s="7">
-        <v>2</v>
-      </c>
-      <c r="J18" s="9">
-        <v>2</v>
-      </c>
-      <c r="K18" s="7">
-        <v>1</v>
+      <c r="H18" s="6">
+        <v>1</v>
+      </c>
+      <c r="I18" s="6">
+        <v>1</v>
+      </c>
+      <c r="J18" s="6">
+        <v>3</v>
+      </c>
+      <c r="K18" s="6">
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2244,32 +2189,32 @@
       <c r="B19" s="6">
         <v>1</v>
       </c>
-      <c r="C19" s="7">
-        <v>2</v>
-      </c>
-      <c r="D19" s="8">
-        <v>0</v>
-      </c>
-      <c r="E19" s="9">
-        <v>4</v>
-      </c>
-      <c r="F19" s="10">
+      <c r="C19" s="6">
+        <v>2</v>
+      </c>
+      <c r="D19" s="6">
+        <v>3</v>
+      </c>
+      <c r="E19" s="6">
+        <v>1</v>
+      </c>
+      <c r="F19" s="6">
         <v>1</v>
       </c>
       <c r="G19" s="6">
         <v>3</v>
       </c>
-      <c r="H19" s="9">
-        <v>1</v>
-      </c>
-      <c r="I19" s="7">
-        <v>2</v>
-      </c>
-      <c r="J19" s="9">
-        <v>2</v>
-      </c>
-      <c r="K19" s="7">
-        <v>1</v>
+      <c r="H19" s="6">
+        <v>3</v>
+      </c>
+      <c r="I19" s="6">
+        <v>2</v>
+      </c>
+      <c r="J19" s="6">
+        <v>3</v>
+      </c>
+      <c r="K19" s="6">
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2279,32 +2224,32 @@
       <c r="B20" s="6">
         <v>1</v>
       </c>
-      <c r="C20" s="7">
-        <v>2</v>
-      </c>
-      <c r="D20" s="8">
-        <v>3</v>
-      </c>
-      <c r="E20" s="9">
-        <v>1</v>
-      </c>
-      <c r="F20" s="10">
-        <v>1</v>
+      <c r="C20" s="6">
+        <v>2</v>
+      </c>
+      <c r="D20" s="6">
+        <v>1</v>
+      </c>
+      <c r="E20" s="6">
+        <v>1</v>
+      </c>
+      <c r="F20" s="6">
+        <v>2</v>
       </c>
       <c r="G20" s="6">
         <v>3</v>
       </c>
-      <c r="H20" s="9">
-        <v>2</v>
-      </c>
-      <c r="I20" s="7">
-        <v>3</v>
-      </c>
-      <c r="J20" s="9">
-        <v>1</v>
-      </c>
-      <c r="K20" s="7">
-        <v>2</v>
+      <c r="H20" s="6">
+        <v>1</v>
+      </c>
+      <c r="I20" s="6">
+        <v>1</v>
+      </c>
+      <c r="J20" s="6">
+        <v>0</v>
+      </c>
+      <c r="K20" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2314,32 +2259,32 @@
       <c r="B21" s="6">
         <v>0</v>
       </c>
-      <c r="C21" s="7">
-        <v>2</v>
-      </c>
-      <c r="D21" s="8">
-        <v>3</v>
-      </c>
-      <c r="E21" s="9">
-        <v>1</v>
-      </c>
-      <c r="F21" s="10">
+      <c r="C21" s="6">
+        <v>4</v>
+      </c>
+      <c r="D21" s="6">
+        <v>1</v>
+      </c>
+      <c r="E21" s="6">
+        <v>1</v>
+      </c>
+      <c r="F21" s="6">
         <v>2</v>
       </c>
       <c r="G21" s="6">
         <v>2</v>
       </c>
-      <c r="H21" s="9">
-        <v>3</v>
-      </c>
-      <c r="I21" s="7">
-        <v>4</v>
-      </c>
-      <c r="J21" s="9">
-        <v>2</v>
-      </c>
-      <c r="K21" s="7">
-        <v>2</v>
+      <c r="H21" s="6">
+        <v>2</v>
+      </c>
+      <c r="I21" s="6">
+        <v>0</v>
+      </c>
+      <c r="J21" s="6">
+        <v>1</v>
+      </c>
+      <c r="K21" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2349,31 +2294,31 @@
       <c r="B22" s="6">
         <v>0</v>
       </c>
-      <c r="C22" s="7">
-        <v>1</v>
-      </c>
-      <c r="D22" s="8">
-        <v>3</v>
-      </c>
-      <c r="E22" s="9">
-        <v>3</v>
-      </c>
-      <c r="F22" s="10">
-        <v>2</v>
+      <c r="C22" s="6">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6">
+        <v>2</v>
+      </c>
+      <c r="E22" s="6">
+        <v>2</v>
+      </c>
+      <c r="F22" s="6">
+        <v>3</v>
       </c>
       <c r="G22" s="6">
         <v>3</v>
       </c>
-      <c r="H22" s="9">
-        <v>2</v>
-      </c>
-      <c r="I22" s="7">
-        <v>2</v>
-      </c>
-      <c r="J22" s="9">
-        <v>1</v>
-      </c>
-      <c r="K22" s="7">
+      <c r="H22" s="6">
+        <v>0</v>
+      </c>
+      <c r="I22" s="6">
+        <v>2</v>
+      </c>
+      <c r="J22" s="6">
+        <v>1</v>
+      </c>
+      <c r="K22" s="6">
         <v>3</v>
       </c>
     </row>
@@ -2384,32 +2329,32 @@
       <c r="B23" s="6">
         <v>0</v>
       </c>
-      <c r="C23" s="7">
-        <v>1</v>
-      </c>
-      <c r="D23" s="8">
-        <v>3</v>
-      </c>
-      <c r="E23" s="9">
-        <v>3</v>
-      </c>
-      <c r="F23" s="10">
+      <c r="C23" s="6">
+        <v>1</v>
+      </c>
+      <c r="D23" s="6">
+        <v>4</v>
+      </c>
+      <c r="E23" s="6">
+        <v>2</v>
+      </c>
+      <c r="F23" s="6">
         <v>1</v>
       </c>
       <c r="G23" s="6">
         <v>4</v>
       </c>
-      <c r="H23" s="9">
-        <v>1</v>
-      </c>
-      <c r="I23" s="7">
-        <v>2</v>
-      </c>
-      <c r="J23" s="9">
-        <v>2</v>
-      </c>
-      <c r="K23" s="7">
-        <v>2</v>
+      <c r="H23" s="6">
+        <v>0</v>
+      </c>
+      <c r="I23" s="6">
+        <v>2</v>
+      </c>
+      <c r="J23" s="6">
+        <v>3</v>
+      </c>
+      <c r="K23" s="6">
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2419,32 +2364,32 @@
       <c r="B24" s="6">
         <v>0</v>
       </c>
-      <c r="C24" s="7">
-        <v>2</v>
-      </c>
-      <c r="D24" s="8">
-        <v>0</v>
-      </c>
-      <c r="E24" s="9">
-        <v>2</v>
-      </c>
-      <c r="F24" s="10">
+      <c r="C24" s="6">
+        <v>3</v>
+      </c>
+      <c r="D24" s="6">
+        <v>3</v>
+      </c>
+      <c r="E24" s="6">
+        <v>0</v>
+      </c>
+      <c r="F24" s="6">
         <v>0</v>
       </c>
       <c r="G24" s="6">
         <v>3</v>
       </c>
-      <c r="H24" s="9">
-        <v>1</v>
-      </c>
-      <c r="I24" s="7">
-        <v>3</v>
-      </c>
-      <c r="J24" s="9">
-        <v>2</v>
-      </c>
-      <c r="K24" s="7">
-        <v>1</v>
+      <c r="H24" s="6">
+        <v>2</v>
+      </c>
+      <c r="I24" s="6">
+        <v>1</v>
+      </c>
+      <c r="J24" s="6">
+        <v>4</v>
+      </c>
+      <c r="K24" s="6">
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -2454,32 +2399,32 @@
       <c r="B25" s="6">
         <v>0</v>
       </c>
-      <c r="C25" s="7">
-        <v>1</v>
-      </c>
-      <c r="D25" s="8">
-        <v>2</v>
-      </c>
-      <c r="E25" s="9">
-        <v>3</v>
-      </c>
-      <c r="F25" s="10">
+      <c r="C25" s="6">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6">
+        <v>4</v>
+      </c>
+      <c r="E25" s="6">
+        <v>1</v>
+      </c>
+      <c r="F25" s="6">
         <v>2</v>
       </c>
       <c r="G25" s="6">
         <v>4</v>
       </c>
-      <c r="H25" s="9">
-        <v>1</v>
-      </c>
-      <c r="I25" s="7">
-        <v>2</v>
-      </c>
-      <c r="J25" s="9">
+      <c r="H25" s="6">
+        <v>1</v>
+      </c>
+      <c r="I25" s="6">
+        <v>2</v>
+      </c>
+      <c r="J25" s="6">
         <v>4</v>
       </c>
-      <c r="K25" s="7">
-        <v>2</v>
+      <c r="K25" s="6">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>